<commit_message>
Add trust & verification, financial tools, WhatsApp OTP phone verification
</commit_message>
<xml_diff>
--- a/public/templates/HyderabadNow_Bulk_Project_Upload_Template.xlsx
+++ b/public/templates/HyderabadNow_Bulk_Project_Upload_Template.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C45"/>
+  <dimension ref="B2:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -888,118 +888,130 @@
     <row r="36">
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>RERA Approval Year</t>
+          <t>RERA Registration Number</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Year — e.g. 2024.</t>
+          <t>Text — e.g. "P02400001234" — shown on the public page with a link to verify it on rera.telangana.gov.in. Leave blank if not yet registered.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Possession Year</t>
+          <t>RERA Approval Year</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Year — Expected/actual handover year.</t>
+          <t>Year — e.g. 2024.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Unit Density Per Acre</t>
+          <t>Possession Year</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Whole number — Units per acre, if known.</t>
+          <t>Year — Expected/actual handover year.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Floor Area Ratio (FAR)</t>
+          <t>Unit Density Per Acre</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Number — e.g. 2.5.</t>
+          <t>Whole number — Units per acre, if known.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Floor Area Ratio (FAR)</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Long text — A paragraph or two about the project.</t>
+          <t>Number — e.g. 2.5.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Amenities</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Comma list of keys — See the 'Amenity Keys' sheet, e.g. "pool,gym,security".</t>
+          <t>Long text — A paragraph or two about the project.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Brochure URL</t>
+          <t>Amenities</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>URL — Link to a hosted brochure PDF, if any.</t>
+          <t>Comma list of keys — See the 'Amenity Keys' sheet, e.g. "pool,gym,security".</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>YouTube Video Link</t>
+          <t>Brochure URL</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>URL — YouTube or Vimeo only.</t>
+          <t>URL — Link to a hosted brochure PDF, if any.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Contact Phone</t>
+          <t>YouTube Video Link</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Text — Sales desk number for the project.</t>
+          <t>URL — YouTube or Vimeo only.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="7" t="inlineStr">
         <is>
+          <t>Contact Phone</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Text — Sales desk number for the project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="7" t="inlineStr">
+        <is>
           <t>Enable WhatsApp Button</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>Dropdown — Yes / No — needs Contact Phone filled in to take effect.</t>
         </is>
@@ -1019,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y202"/>
+  <dimension ref="A1:Z202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1037,16 +1049,17 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="34" customWidth="1" min="20" max="20"/>
-    <col width="26" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
-    <col width="24" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
@@ -1127,50 +1140,55 @@
       </c>
       <c r="P1" s="9" t="inlineStr">
         <is>
+          <t>RERA Registration Number</t>
+        </is>
+      </c>
+      <c r="Q1" s="9" t="inlineStr">
+        <is>
           <t>RERA Approval Year</t>
         </is>
       </c>
-      <c r="Q1" s="9" t="inlineStr">
+      <c r="R1" s="9" t="inlineStr">
         <is>
           <t>Possession Year</t>
         </is>
       </c>
-      <c r="R1" s="9" t="inlineStr">
+      <c r="S1" s="9" t="inlineStr">
         <is>
           <t>Unit Density Per Acre</t>
         </is>
       </c>
-      <c r="S1" s="9" t="inlineStr">
+      <c r="T1" s="9" t="inlineStr">
         <is>
           <t>Floor Area Ratio (FAR)</t>
         </is>
       </c>
-      <c r="T1" s="9" t="inlineStr">
+      <c r="U1" s="9" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="U1" s="9" t="inlineStr">
+      <c r="V1" s="9" t="inlineStr">
         <is>
           <t>Amenities</t>
         </is>
       </c>
-      <c r="V1" s="9" t="inlineStr">
+      <c r="W1" s="9" t="inlineStr">
         <is>
           <t>Brochure URL</t>
         </is>
       </c>
-      <c r="W1" s="9" t="inlineStr">
+      <c r="X1" s="9" t="inlineStr">
         <is>
           <t>YouTube Video Link</t>
         </is>
       </c>
-      <c r="X1" s="9" t="inlineStr">
+      <c r="Y1" s="9" t="inlineStr">
         <is>
           <t>Contact Phone</t>
         </is>
       </c>
-      <c r="Y1" s="9" t="inlineStr">
+      <c r="Z1" s="9" t="inlineStr">
         <is>
           <t>Enable WhatsApp Button</t>
         </is>
@@ -1240,44 +1258,49 @@
           <t>2,2.5,3</t>
         </is>
       </c>
-      <c r="P2" s="10" t="n">
+      <c r="P2" s="10" t="inlineStr">
+        <is>
+          <t>P02400001234</t>
+        </is>
+      </c>
+      <c r="Q2" s="10" t="n">
         <v>2024</v>
       </c>
-      <c r="Q2" s="10" t="n">
+      <c r="R2" s="10" t="n">
         <v>2028</v>
       </c>
-      <c r="R2" s="10" t="n">
+      <c r="S2" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="S2" s="10" t="n">
+      <c r="T2" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="T2" s="10" t="inlineStr">
+      <c r="U2" s="10" t="inlineStr">
         <is>
           <t>A gated high-rise community with landscaped courtyards, close to the Financial District and the ORR.</t>
         </is>
       </c>
-      <c r="U2" s="10" t="inlineStr">
+      <c r="V2" s="10" t="inlineStr">
         <is>
           <t>pool,gym,clubhouse,security,lift,parking</t>
         </is>
       </c>
-      <c r="V2" s="10" t="inlineStr">
+      <c r="W2" s="10" t="inlineStr">
         <is>
           <t>https://example.com/brochure.pdf</t>
         </is>
       </c>
-      <c r="W2" s="10" t="inlineStr">
+      <c r="X2" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=example</t>
         </is>
       </c>
-      <c r="X2" s="10" t="inlineStr">
+      <c r="Y2" s="10" t="inlineStr">
         <is>
           <t>+91 90000 00000</t>
         </is>
       </c>
-      <c r="Y2" s="10" t="inlineStr">
+      <c r="Z2" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1309,6 +1332,7 @@
       <c r="W3" s="11" t="n"/>
       <c r="X3" s="11" t="n"/>
       <c r="Y3" s="11" t="n"/>
+      <c r="Z3" s="11" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="n"/>
@@ -1336,6 +1360,7 @@
       <c r="W4" s="11" t="n"/>
       <c r="X4" s="11" t="n"/>
       <c r="Y4" s="11" t="n"/>
+      <c r="Z4" s="11" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="n"/>
@@ -1363,6 +1388,7 @@
       <c r="W5" s="11" t="n"/>
       <c r="X5" s="11" t="n"/>
       <c r="Y5" s="11" t="n"/>
+      <c r="Z5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n"/>
@@ -1390,6 +1416,7 @@
       <c r="W6" s="11" t="n"/>
       <c r="X6" s="11" t="n"/>
       <c r="Y6" s="11" t="n"/>
+      <c r="Z6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n"/>
@@ -1417,6 +1444,7 @@
       <c r="W7" s="11" t="n"/>
       <c r="X7" s="11" t="n"/>
       <c r="Y7" s="11" t="n"/>
+      <c r="Z7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="n"/>
@@ -1444,6 +1472,7 @@
       <c r="W8" s="11" t="n"/>
       <c r="X8" s="11" t="n"/>
       <c r="Y8" s="11" t="n"/>
+      <c r="Z8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="n"/>
@@ -1471,6 +1500,7 @@
       <c r="W9" s="11" t="n"/>
       <c r="X9" s="11" t="n"/>
       <c r="Y9" s="11" t="n"/>
+      <c r="Z9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n"/>
@@ -1498,6 +1528,7 @@
       <c r="W10" s="11" t="n"/>
       <c r="X10" s="11" t="n"/>
       <c r="Y10" s="11" t="n"/>
+      <c r="Z10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n"/>
@@ -1525,6 +1556,7 @@
       <c r="W11" s="11" t="n"/>
       <c r="X11" s="11" t="n"/>
       <c r="Y11" s="11" t="n"/>
+      <c r="Z11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n"/>
@@ -1552,6 +1584,7 @@
       <c r="W12" s="11" t="n"/>
       <c r="X12" s="11" t="n"/>
       <c r="Y12" s="11" t="n"/>
+      <c r="Z12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n"/>
@@ -1579,6 +1612,7 @@
       <c r="W13" s="11" t="n"/>
       <c r="X13" s="11" t="n"/>
       <c r="Y13" s="11" t="n"/>
+      <c r="Z13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="n"/>
@@ -1606,6 +1640,7 @@
       <c r="W14" s="11" t="n"/>
       <c r="X14" s="11" t="n"/>
       <c r="Y14" s="11" t="n"/>
+      <c r="Z14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n"/>
@@ -1633,6 +1668,7 @@
       <c r="W15" s="11" t="n"/>
       <c r="X15" s="11" t="n"/>
       <c r="Y15" s="11" t="n"/>
+      <c r="Z15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="n"/>
@@ -1660,6 +1696,7 @@
       <c r="W16" s="11" t="n"/>
       <c r="X16" s="11" t="n"/>
       <c r="Y16" s="11" t="n"/>
+      <c r="Z16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n"/>
@@ -1687,6 +1724,7 @@
       <c r="W17" s="11" t="n"/>
       <c r="X17" s="11" t="n"/>
       <c r="Y17" s="11" t="n"/>
+      <c r="Z17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n"/>
@@ -1714,6 +1752,7 @@
       <c r="W18" s="11" t="n"/>
       <c r="X18" s="11" t="n"/>
       <c r="Y18" s="11" t="n"/>
+      <c r="Z18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n"/>
@@ -1741,6 +1780,7 @@
       <c r="W19" s="11" t="n"/>
       <c r="X19" s="11" t="n"/>
       <c r="Y19" s="11" t="n"/>
+      <c r="Z19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="11" t="n"/>
@@ -1768,6 +1808,7 @@
       <c r="W20" s="11" t="n"/>
       <c r="X20" s="11" t="n"/>
       <c r="Y20" s="11" t="n"/>
+      <c r="Z20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n"/>
@@ -1795,6 +1836,7 @@
       <c r="W21" s="11" t="n"/>
       <c r="X21" s="11" t="n"/>
       <c r="Y21" s="11" t="n"/>
+      <c r="Z21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n"/>
@@ -1822,6 +1864,7 @@
       <c r="W22" s="11" t="n"/>
       <c r="X22" s="11" t="n"/>
       <c r="Y22" s="11" t="n"/>
+      <c r="Z22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n"/>
@@ -1849,6 +1892,7 @@
       <c r="W23" s="11" t="n"/>
       <c r="X23" s="11" t="n"/>
       <c r="Y23" s="11" t="n"/>
+      <c r="Z23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n"/>
@@ -1876,6 +1920,7 @@
       <c r="W24" s="11" t="n"/>
       <c r="X24" s="11" t="n"/>
       <c r="Y24" s="11" t="n"/>
+      <c r="Z24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n"/>
@@ -1903,6 +1948,7 @@
       <c r="W25" s="11" t="n"/>
       <c r="X25" s="11" t="n"/>
       <c r="Y25" s="11" t="n"/>
+      <c r="Z25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n"/>
@@ -1930,6 +1976,7 @@
       <c r="W26" s="11" t="n"/>
       <c r="X26" s="11" t="n"/>
       <c r="Y26" s="11" t="n"/>
+      <c r="Z26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n"/>
@@ -1957,6 +2004,7 @@
       <c r="W27" s="11" t="n"/>
       <c r="X27" s="11" t="n"/>
       <c r="Y27" s="11" t="n"/>
+      <c r="Z27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n"/>
@@ -1984,6 +2032,7 @@
       <c r="W28" s="11" t="n"/>
       <c r="X28" s="11" t="n"/>
       <c r="Y28" s="11" t="n"/>
+      <c r="Z28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n"/>
@@ -2011,6 +2060,7 @@
       <c r="W29" s="11" t="n"/>
       <c r="X29" s="11" t="n"/>
       <c r="Y29" s="11" t="n"/>
+      <c r="Z29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n"/>
@@ -2038,6 +2088,7 @@
       <c r="W30" s="11" t="n"/>
       <c r="X30" s="11" t="n"/>
       <c r="Y30" s="11" t="n"/>
+      <c r="Z30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n"/>
@@ -2065,6 +2116,7 @@
       <c r="W31" s="11" t="n"/>
       <c r="X31" s="11" t="n"/>
       <c r="Y31" s="11" t="n"/>
+      <c r="Z31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n"/>
@@ -2092,6 +2144,7 @@
       <c r="W32" s="11" t="n"/>
       <c r="X32" s="11" t="n"/>
       <c r="Y32" s="11" t="n"/>
+      <c r="Z32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n"/>
@@ -2119,6 +2172,7 @@
       <c r="W33" s="11" t="n"/>
       <c r="X33" s="11" t="n"/>
       <c r="Y33" s="11" t="n"/>
+      <c r="Z33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n"/>
@@ -2146,6 +2200,7 @@
       <c r="W34" s="11" t="n"/>
       <c r="X34" s="11" t="n"/>
       <c r="Y34" s="11" t="n"/>
+      <c r="Z34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n"/>
@@ -2173,6 +2228,7 @@
       <c r="W35" s="11" t="n"/>
       <c r="X35" s="11" t="n"/>
       <c r="Y35" s="11" t="n"/>
+      <c r="Z35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n"/>
@@ -2200,6 +2256,7 @@
       <c r="W36" s="11" t="n"/>
       <c r="X36" s="11" t="n"/>
       <c r="Y36" s="11" t="n"/>
+      <c r="Z36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n"/>
@@ -2227,6 +2284,7 @@
       <c r="W37" s="11" t="n"/>
       <c r="X37" s="11" t="n"/>
       <c r="Y37" s="11" t="n"/>
+      <c r="Z37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n"/>
@@ -2254,6 +2312,7 @@
       <c r="W38" s="11" t="n"/>
       <c r="X38" s="11" t="n"/>
       <c r="Y38" s="11" t="n"/>
+      <c r="Z38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n"/>
@@ -2281,6 +2340,7 @@
       <c r="W39" s="11" t="n"/>
       <c r="X39" s="11" t="n"/>
       <c r="Y39" s="11" t="n"/>
+      <c r="Z39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n"/>
@@ -2308,6 +2368,7 @@
       <c r="W40" s="11" t="n"/>
       <c r="X40" s="11" t="n"/>
       <c r="Y40" s="11" t="n"/>
+      <c r="Z40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n"/>
@@ -2335,6 +2396,7 @@
       <c r="W41" s="11" t="n"/>
       <c r="X41" s="11" t="n"/>
       <c r="Y41" s="11" t="n"/>
+      <c r="Z41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n"/>
@@ -2362,6 +2424,7 @@
       <c r="W42" s="11" t="n"/>
       <c r="X42" s="11" t="n"/>
       <c r="Y42" s="11" t="n"/>
+      <c r="Z42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="11" t="n"/>
@@ -2389,6 +2452,7 @@
       <c r="W43" s="11" t="n"/>
       <c r="X43" s="11" t="n"/>
       <c r="Y43" s="11" t="n"/>
+      <c r="Z43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n"/>
@@ -2416,6 +2480,7 @@
       <c r="W44" s="11" t="n"/>
       <c r="X44" s="11" t="n"/>
       <c r="Y44" s="11" t="n"/>
+      <c r="Z44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n"/>
@@ -2443,6 +2508,7 @@
       <c r="W45" s="11" t="n"/>
       <c r="X45" s="11" t="n"/>
       <c r="Y45" s="11" t="n"/>
+      <c r="Z45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n"/>
@@ -2470,6 +2536,7 @@
       <c r="W46" s="11" t="n"/>
       <c r="X46" s="11" t="n"/>
       <c r="Y46" s="11" t="n"/>
+      <c r="Z46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="11" t="n"/>
@@ -2497,6 +2564,7 @@
       <c r="W47" s="11" t="n"/>
       <c r="X47" s="11" t="n"/>
       <c r="Y47" s="11" t="n"/>
+      <c r="Z47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="11" t="n"/>
@@ -2524,6 +2592,7 @@
       <c r="W48" s="11" t="n"/>
       <c r="X48" s="11" t="n"/>
       <c r="Y48" s="11" t="n"/>
+      <c r="Z48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="11" t="n"/>
@@ -2551,6 +2620,7 @@
       <c r="W49" s="11" t="n"/>
       <c r="X49" s="11" t="n"/>
       <c r="Y49" s="11" t="n"/>
+      <c r="Z49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n"/>
@@ -2578,6 +2648,7 @@
       <c r="W50" s="11" t="n"/>
       <c r="X50" s="11" t="n"/>
       <c r="Y50" s="11" t="n"/>
+      <c r="Z50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n"/>
@@ -2605,6 +2676,7 @@
       <c r="W51" s="11" t="n"/>
       <c r="X51" s="11" t="n"/>
       <c r="Y51" s="11" t="n"/>
+      <c r="Z51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n"/>
@@ -2632,6 +2704,7 @@
       <c r="W52" s="11" t="n"/>
       <c r="X52" s="11" t="n"/>
       <c r="Y52" s="11" t="n"/>
+      <c r="Z52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n"/>
@@ -2659,6 +2732,7 @@
       <c r="W53" s="11" t="n"/>
       <c r="X53" s="11" t="n"/>
       <c r="Y53" s="11" t="n"/>
+      <c r="Z53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n"/>
@@ -2686,6 +2760,7 @@
       <c r="W54" s="11" t="n"/>
       <c r="X54" s="11" t="n"/>
       <c r="Y54" s="11" t="n"/>
+      <c r="Z54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n"/>
@@ -2713,6 +2788,7 @@
       <c r="W55" s="11" t="n"/>
       <c r="X55" s="11" t="n"/>
       <c r="Y55" s="11" t="n"/>
+      <c r="Z55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n"/>
@@ -2740,6 +2816,7 @@
       <c r="W56" s="11" t="n"/>
       <c r="X56" s="11" t="n"/>
       <c r="Y56" s="11" t="n"/>
+      <c r="Z56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n"/>
@@ -2767,6 +2844,7 @@
       <c r="W57" s="11" t="n"/>
       <c r="X57" s="11" t="n"/>
       <c r="Y57" s="11" t="n"/>
+      <c r="Z57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n"/>
@@ -2794,6 +2872,7 @@
       <c r="W58" s="11" t="n"/>
       <c r="X58" s="11" t="n"/>
       <c r="Y58" s="11" t="n"/>
+      <c r="Z58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n"/>
@@ -2821,6 +2900,7 @@
       <c r="W59" s="11" t="n"/>
       <c r="X59" s="11" t="n"/>
       <c r="Y59" s="11" t="n"/>
+      <c r="Z59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n"/>
@@ -2848,6 +2928,7 @@
       <c r="W60" s="11" t="n"/>
       <c r="X60" s="11" t="n"/>
       <c r="Y60" s="11" t="n"/>
+      <c r="Z60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n"/>
@@ -2875,6 +2956,7 @@
       <c r="W61" s="11" t="n"/>
       <c r="X61" s="11" t="n"/>
       <c r="Y61" s="11" t="n"/>
+      <c r="Z61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n"/>
@@ -2902,6 +2984,7 @@
       <c r="W62" s="11" t="n"/>
       <c r="X62" s="11" t="n"/>
       <c r="Y62" s="11" t="n"/>
+      <c r="Z62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n"/>
@@ -2929,6 +3012,7 @@
       <c r="W63" s="11" t="n"/>
       <c r="X63" s="11" t="n"/>
       <c r="Y63" s="11" t="n"/>
+      <c r="Z63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n"/>
@@ -2956,6 +3040,7 @@
       <c r="W64" s="11" t="n"/>
       <c r="X64" s="11" t="n"/>
       <c r="Y64" s="11" t="n"/>
+      <c r="Z64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n"/>
@@ -2983,6 +3068,7 @@
       <c r="W65" s="11" t="n"/>
       <c r="X65" s="11" t="n"/>
       <c r="Y65" s="11" t="n"/>
+      <c r="Z65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="11" t="n"/>
@@ -3010,6 +3096,7 @@
       <c r="W66" s="11" t="n"/>
       <c r="X66" s="11" t="n"/>
       <c r="Y66" s="11" t="n"/>
+      <c r="Z66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n"/>
@@ -3037,6 +3124,7 @@
       <c r="W67" s="11" t="n"/>
       <c r="X67" s="11" t="n"/>
       <c r="Y67" s="11" t="n"/>
+      <c r="Z67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="11" t="n"/>
@@ -3064,6 +3152,7 @@
       <c r="W68" s="11" t="n"/>
       <c r="X68" s="11" t="n"/>
       <c r="Y68" s="11" t="n"/>
+      <c r="Z68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="n"/>
@@ -3091,6 +3180,7 @@
       <c r="W69" s="11" t="n"/>
       <c r="X69" s="11" t="n"/>
       <c r="Y69" s="11" t="n"/>
+      <c r="Z69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="n"/>
@@ -3118,6 +3208,7 @@
       <c r="W70" s="11" t="n"/>
       <c r="X70" s="11" t="n"/>
       <c r="Y70" s="11" t="n"/>
+      <c r="Z70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="11" t="n"/>
@@ -3145,6 +3236,7 @@
       <c r="W71" s="11" t="n"/>
       <c r="X71" s="11" t="n"/>
       <c r="Y71" s="11" t="n"/>
+      <c r="Z71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="11" t="n"/>
@@ -3172,6 +3264,7 @@
       <c r="W72" s="11" t="n"/>
       <c r="X72" s="11" t="n"/>
       <c r="Y72" s="11" t="n"/>
+      <c r="Z72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="11" t="n"/>
@@ -3199,6 +3292,7 @@
       <c r="W73" s="11" t="n"/>
       <c r="X73" s="11" t="n"/>
       <c r="Y73" s="11" t="n"/>
+      <c r="Z73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="11" t="n"/>
@@ -3226,6 +3320,7 @@
       <c r="W74" s="11" t="n"/>
       <c r="X74" s="11" t="n"/>
       <c r="Y74" s="11" t="n"/>
+      <c r="Z74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="11" t="n"/>
@@ -3253,6 +3348,7 @@
       <c r="W75" s="11" t="n"/>
       <c r="X75" s="11" t="n"/>
       <c r="Y75" s="11" t="n"/>
+      <c r="Z75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="11" t="n"/>
@@ -3280,6 +3376,7 @@
       <c r="W76" s="11" t="n"/>
       <c r="X76" s="11" t="n"/>
       <c r="Y76" s="11" t="n"/>
+      <c r="Z76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="11" t="n"/>
@@ -3307,6 +3404,7 @@
       <c r="W77" s="11" t="n"/>
       <c r="X77" s="11" t="n"/>
       <c r="Y77" s="11" t="n"/>
+      <c r="Z77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="11" t="n"/>
@@ -3334,6 +3432,7 @@
       <c r="W78" s="11" t="n"/>
       <c r="X78" s="11" t="n"/>
       <c r="Y78" s="11" t="n"/>
+      <c r="Z78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="11" t="n"/>
@@ -3361,6 +3460,7 @@
       <c r="W79" s="11" t="n"/>
       <c r="X79" s="11" t="n"/>
       <c r="Y79" s="11" t="n"/>
+      <c r="Z79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="11" t="n"/>
@@ -3388,6 +3488,7 @@
       <c r="W80" s="11" t="n"/>
       <c r="X80" s="11" t="n"/>
       <c r="Y80" s="11" t="n"/>
+      <c r="Z80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="11" t="n"/>
@@ -3415,6 +3516,7 @@
       <c r="W81" s="11" t="n"/>
       <c r="X81" s="11" t="n"/>
       <c r="Y81" s="11" t="n"/>
+      <c r="Z81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="11" t="n"/>
@@ -3442,6 +3544,7 @@
       <c r="W82" s="11" t="n"/>
       <c r="X82" s="11" t="n"/>
       <c r="Y82" s="11" t="n"/>
+      <c r="Z82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="11" t="n"/>
@@ -3469,6 +3572,7 @@
       <c r="W83" s="11" t="n"/>
       <c r="X83" s="11" t="n"/>
       <c r="Y83" s="11" t="n"/>
+      <c r="Z83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="11" t="n"/>
@@ -3496,6 +3600,7 @@
       <c r="W84" s="11" t="n"/>
       <c r="X84" s="11" t="n"/>
       <c r="Y84" s="11" t="n"/>
+      <c r="Z84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="11" t="n"/>
@@ -3523,6 +3628,7 @@
       <c r="W85" s="11" t="n"/>
       <c r="X85" s="11" t="n"/>
       <c r="Y85" s="11" t="n"/>
+      <c r="Z85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="11" t="n"/>
@@ -3550,6 +3656,7 @@
       <c r="W86" s="11" t="n"/>
       <c r="X86" s="11" t="n"/>
       <c r="Y86" s="11" t="n"/>
+      <c r="Z86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="11" t="n"/>
@@ -3577,6 +3684,7 @@
       <c r="W87" s="11" t="n"/>
       <c r="X87" s="11" t="n"/>
       <c r="Y87" s="11" t="n"/>
+      <c r="Z87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="11" t="n"/>
@@ -3604,6 +3712,7 @@
       <c r="W88" s="11" t="n"/>
       <c r="X88" s="11" t="n"/>
       <c r="Y88" s="11" t="n"/>
+      <c r="Z88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="11" t="n"/>
@@ -3631,6 +3740,7 @@
       <c r="W89" s="11" t="n"/>
       <c r="X89" s="11" t="n"/>
       <c r="Y89" s="11" t="n"/>
+      <c r="Z89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="11" t="n"/>
@@ -3658,6 +3768,7 @@
       <c r="W90" s="11" t="n"/>
       <c r="X90" s="11" t="n"/>
       <c r="Y90" s="11" t="n"/>
+      <c r="Z90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="11" t="n"/>
@@ -3685,6 +3796,7 @@
       <c r="W91" s="11" t="n"/>
       <c r="X91" s="11" t="n"/>
       <c r="Y91" s="11" t="n"/>
+      <c r="Z91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="11" t="n"/>
@@ -3712,6 +3824,7 @@
       <c r="W92" s="11" t="n"/>
       <c r="X92" s="11" t="n"/>
       <c r="Y92" s="11" t="n"/>
+      <c r="Z92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="11" t="n"/>
@@ -3739,6 +3852,7 @@
       <c r="W93" s="11" t="n"/>
       <c r="X93" s="11" t="n"/>
       <c r="Y93" s="11" t="n"/>
+      <c r="Z93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="11" t="n"/>
@@ -3766,6 +3880,7 @@
       <c r="W94" s="11" t="n"/>
       <c r="X94" s="11" t="n"/>
       <c r="Y94" s="11" t="n"/>
+      <c r="Z94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="11" t="n"/>
@@ -3793,6 +3908,7 @@
       <c r="W95" s="11" t="n"/>
       <c r="X95" s="11" t="n"/>
       <c r="Y95" s="11" t="n"/>
+      <c r="Z95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="11" t="n"/>
@@ -3820,6 +3936,7 @@
       <c r="W96" s="11" t="n"/>
       <c r="X96" s="11" t="n"/>
       <c r="Y96" s="11" t="n"/>
+      <c r="Z96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="11" t="n"/>
@@ -3847,6 +3964,7 @@
       <c r="W97" s="11" t="n"/>
       <c r="X97" s="11" t="n"/>
       <c r="Y97" s="11" t="n"/>
+      <c r="Z97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="11" t="n"/>
@@ -3874,6 +3992,7 @@
       <c r="W98" s="11" t="n"/>
       <c r="X98" s="11" t="n"/>
       <c r="Y98" s="11" t="n"/>
+      <c r="Z98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="11" t="n"/>
@@ -3901,6 +4020,7 @@
       <c r="W99" s="11" t="n"/>
       <c r="X99" s="11" t="n"/>
       <c r="Y99" s="11" t="n"/>
+      <c r="Z99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="11" t="n"/>
@@ -3928,6 +4048,7 @@
       <c r="W100" s="11" t="n"/>
       <c r="X100" s="11" t="n"/>
       <c r="Y100" s="11" t="n"/>
+      <c r="Z100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="11" t="n"/>
@@ -3955,6 +4076,7 @@
       <c r="W101" s="11" t="n"/>
       <c r="X101" s="11" t="n"/>
       <c r="Y101" s="11" t="n"/>
+      <c r="Z101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="11" t="n"/>
@@ -3982,6 +4104,7 @@
       <c r="W102" s="11" t="n"/>
       <c r="X102" s="11" t="n"/>
       <c r="Y102" s="11" t="n"/>
+      <c r="Z102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="11" t="n"/>
@@ -4009,6 +4132,7 @@
       <c r="W103" s="11" t="n"/>
       <c r="X103" s="11" t="n"/>
       <c r="Y103" s="11" t="n"/>
+      <c r="Z103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="11" t="n"/>
@@ -4036,6 +4160,7 @@
       <c r="W104" s="11" t="n"/>
       <c r="X104" s="11" t="n"/>
       <c r="Y104" s="11" t="n"/>
+      <c r="Z104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="11" t="n"/>
@@ -4063,6 +4188,7 @@
       <c r="W105" s="11" t="n"/>
       <c r="X105" s="11" t="n"/>
       <c r="Y105" s="11" t="n"/>
+      <c r="Z105" s="11" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="11" t="n"/>
@@ -4090,6 +4216,7 @@
       <c r="W106" s="11" t="n"/>
       <c r="X106" s="11" t="n"/>
       <c r="Y106" s="11" t="n"/>
+      <c r="Z106" s="11" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="11" t="n"/>
@@ -4117,6 +4244,7 @@
       <c r="W107" s="11" t="n"/>
       <c r="X107" s="11" t="n"/>
       <c r="Y107" s="11" t="n"/>
+      <c r="Z107" s="11" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="11" t="n"/>
@@ -4144,6 +4272,7 @@
       <c r="W108" s="11" t="n"/>
       <c r="X108" s="11" t="n"/>
       <c r="Y108" s="11" t="n"/>
+      <c r="Z108" s="11" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="11" t="n"/>
@@ -4171,6 +4300,7 @@
       <c r="W109" s="11" t="n"/>
       <c r="X109" s="11" t="n"/>
       <c r="Y109" s="11" t="n"/>
+      <c r="Z109" s="11" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="11" t="n"/>
@@ -4198,6 +4328,7 @@
       <c r="W110" s="11" t="n"/>
       <c r="X110" s="11" t="n"/>
       <c r="Y110" s="11" t="n"/>
+      <c r="Z110" s="11" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="11" t="n"/>
@@ -4225,6 +4356,7 @@
       <c r="W111" s="11" t="n"/>
       <c r="X111" s="11" t="n"/>
       <c r="Y111" s="11" t="n"/>
+      <c r="Z111" s="11" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="11" t="n"/>
@@ -4252,6 +4384,7 @@
       <c r="W112" s="11" t="n"/>
       <c r="X112" s="11" t="n"/>
       <c r="Y112" s="11" t="n"/>
+      <c r="Z112" s="11" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="11" t="n"/>
@@ -4279,6 +4412,7 @@
       <c r="W113" s="11" t="n"/>
       <c r="X113" s="11" t="n"/>
       <c r="Y113" s="11" t="n"/>
+      <c r="Z113" s="11" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="11" t="n"/>
@@ -4306,6 +4440,7 @@
       <c r="W114" s="11" t="n"/>
       <c r="X114" s="11" t="n"/>
       <c r="Y114" s="11" t="n"/>
+      <c r="Z114" s="11" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="11" t="n"/>
@@ -4333,6 +4468,7 @@
       <c r="W115" s="11" t="n"/>
       <c r="X115" s="11" t="n"/>
       <c r="Y115" s="11" t="n"/>
+      <c r="Z115" s="11" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="11" t="n"/>
@@ -4360,6 +4496,7 @@
       <c r="W116" s="11" t="n"/>
       <c r="X116" s="11" t="n"/>
       <c r="Y116" s="11" t="n"/>
+      <c r="Z116" s="11" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="11" t="n"/>
@@ -4387,6 +4524,7 @@
       <c r="W117" s="11" t="n"/>
       <c r="X117" s="11" t="n"/>
       <c r="Y117" s="11" t="n"/>
+      <c r="Z117" s="11" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="11" t="n"/>
@@ -4414,6 +4552,7 @@
       <c r="W118" s="11" t="n"/>
       <c r="X118" s="11" t="n"/>
       <c r="Y118" s="11" t="n"/>
+      <c r="Z118" s="11" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="11" t="n"/>
@@ -4441,6 +4580,7 @@
       <c r="W119" s="11" t="n"/>
       <c r="X119" s="11" t="n"/>
       <c r="Y119" s="11" t="n"/>
+      <c r="Z119" s="11" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="11" t="n"/>
@@ -4468,6 +4608,7 @@
       <c r="W120" s="11" t="n"/>
       <c r="X120" s="11" t="n"/>
       <c r="Y120" s="11" t="n"/>
+      <c r="Z120" s="11" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="11" t="n"/>
@@ -4495,6 +4636,7 @@
       <c r="W121" s="11" t="n"/>
       <c r="X121" s="11" t="n"/>
       <c r="Y121" s="11" t="n"/>
+      <c r="Z121" s="11" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="11" t="n"/>
@@ -4522,6 +4664,7 @@
       <c r="W122" s="11" t="n"/>
       <c r="X122" s="11" t="n"/>
       <c r="Y122" s="11" t="n"/>
+      <c r="Z122" s="11" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="11" t="n"/>
@@ -4549,6 +4692,7 @@
       <c r="W123" s="11" t="n"/>
       <c r="X123" s="11" t="n"/>
       <c r="Y123" s="11" t="n"/>
+      <c r="Z123" s="11" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="11" t="n"/>
@@ -4576,6 +4720,7 @@
       <c r="W124" s="11" t="n"/>
       <c r="X124" s="11" t="n"/>
       <c r="Y124" s="11" t="n"/>
+      <c r="Z124" s="11" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="11" t="n"/>
@@ -4603,6 +4748,7 @@
       <c r="W125" s="11" t="n"/>
       <c r="X125" s="11" t="n"/>
       <c r="Y125" s="11" t="n"/>
+      <c r="Z125" s="11" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="11" t="n"/>
@@ -4630,6 +4776,7 @@
       <c r="W126" s="11" t="n"/>
       <c r="X126" s="11" t="n"/>
       <c r="Y126" s="11" t="n"/>
+      <c r="Z126" s="11" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="11" t="n"/>
@@ -4657,6 +4804,7 @@
       <c r="W127" s="11" t="n"/>
       <c r="X127" s="11" t="n"/>
       <c r="Y127" s="11" t="n"/>
+      <c r="Z127" s="11" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="11" t="n"/>
@@ -4684,6 +4832,7 @@
       <c r="W128" s="11" t="n"/>
       <c r="X128" s="11" t="n"/>
       <c r="Y128" s="11" t="n"/>
+      <c r="Z128" s="11" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="11" t="n"/>
@@ -4711,6 +4860,7 @@
       <c r="W129" s="11" t="n"/>
       <c r="X129" s="11" t="n"/>
       <c r="Y129" s="11" t="n"/>
+      <c r="Z129" s="11" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="11" t="n"/>
@@ -4738,6 +4888,7 @@
       <c r="W130" s="11" t="n"/>
       <c r="X130" s="11" t="n"/>
       <c r="Y130" s="11" t="n"/>
+      <c r="Z130" s="11" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="11" t="n"/>
@@ -4765,6 +4916,7 @@
       <c r="W131" s="11" t="n"/>
       <c r="X131" s="11" t="n"/>
       <c r="Y131" s="11" t="n"/>
+      <c r="Z131" s="11" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="11" t="n"/>
@@ -4792,6 +4944,7 @@
       <c r="W132" s="11" t="n"/>
       <c r="X132" s="11" t="n"/>
       <c r="Y132" s="11" t="n"/>
+      <c r="Z132" s="11" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="11" t="n"/>
@@ -4819,6 +4972,7 @@
       <c r="W133" s="11" t="n"/>
       <c r="X133" s="11" t="n"/>
       <c r="Y133" s="11" t="n"/>
+      <c r="Z133" s="11" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="11" t="n"/>
@@ -4846,6 +5000,7 @@
       <c r="W134" s="11" t="n"/>
       <c r="X134" s="11" t="n"/>
       <c r="Y134" s="11" t="n"/>
+      <c r="Z134" s="11" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="11" t="n"/>
@@ -4873,6 +5028,7 @@
       <c r="W135" s="11" t="n"/>
       <c r="X135" s="11" t="n"/>
       <c r="Y135" s="11" t="n"/>
+      <c r="Z135" s="11" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="11" t="n"/>
@@ -4900,6 +5056,7 @@
       <c r="W136" s="11" t="n"/>
       <c r="X136" s="11" t="n"/>
       <c r="Y136" s="11" t="n"/>
+      <c r="Z136" s="11" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="11" t="n"/>
@@ -4927,6 +5084,7 @@
       <c r="W137" s="11" t="n"/>
       <c r="X137" s="11" t="n"/>
       <c r="Y137" s="11" t="n"/>
+      <c r="Z137" s="11" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="11" t="n"/>
@@ -4954,6 +5112,7 @@
       <c r="W138" s="11" t="n"/>
       <c r="X138" s="11" t="n"/>
       <c r="Y138" s="11" t="n"/>
+      <c r="Z138" s="11" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="11" t="n"/>
@@ -4981,6 +5140,7 @@
       <c r="W139" s="11" t="n"/>
       <c r="X139" s="11" t="n"/>
       <c r="Y139" s="11" t="n"/>
+      <c r="Z139" s="11" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="11" t="n"/>
@@ -5008,6 +5168,7 @@
       <c r="W140" s="11" t="n"/>
       <c r="X140" s="11" t="n"/>
       <c r="Y140" s="11" t="n"/>
+      <c r="Z140" s="11" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="11" t="n"/>
@@ -5035,6 +5196,7 @@
       <c r="W141" s="11" t="n"/>
       <c r="X141" s="11" t="n"/>
       <c r="Y141" s="11" t="n"/>
+      <c r="Z141" s="11" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="11" t="n"/>
@@ -5062,6 +5224,7 @@
       <c r="W142" s="11" t="n"/>
       <c r="X142" s="11" t="n"/>
       <c r="Y142" s="11" t="n"/>
+      <c r="Z142" s="11" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="11" t="n"/>
@@ -5089,6 +5252,7 @@
       <c r="W143" s="11" t="n"/>
       <c r="X143" s="11" t="n"/>
       <c r="Y143" s="11" t="n"/>
+      <c r="Z143" s="11" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="11" t="n"/>
@@ -5116,6 +5280,7 @@
       <c r="W144" s="11" t="n"/>
       <c r="X144" s="11" t="n"/>
       <c r="Y144" s="11" t="n"/>
+      <c r="Z144" s="11" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="11" t="n"/>
@@ -5143,6 +5308,7 @@
       <c r="W145" s="11" t="n"/>
       <c r="X145" s="11" t="n"/>
       <c r="Y145" s="11" t="n"/>
+      <c r="Z145" s="11" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="11" t="n"/>
@@ -5170,6 +5336,7 @@
       <c r="W146" s="11" t="n"/>
       <c r="X146" s="11" t="n"/>
       <c r="Y146" s="11" t="n"/>
+      <c r="Z146" s="11" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="11" t="n"/>
@@ -5197,6 +5364,7 @@
       <c r="W147" s="11" t="n"/>
       <c r="X147" s="11" t="n"/>
       <c r="Y147" s="11" t="n"/>
+      <c r="Z147" s="11" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="11" t="n"/>
@@ -5224,6 +5392,7 @@
       <c r="W148" s="11" t="n"/>
       <c r="X148" s="11" t="n"/>
       <c r="Y148" s="11" t="n"/>
+      <c r="Z148" s="11" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="11" t="n"/>
@@ -5251,6 +5420,7 @@
       <c r="W149" s="11" t="n"/>
       <c r="X149" s="11" t="n"/>
       <c r="Y149" s="11" t="n"/>
+      <c r="Z149" s="11" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="11" t="n"/>
@@ -5278,6 +5448,7 @@
       <c r="W150" s="11" t="n"/>
       <c r="X150" s="11" t="n"/>
       <c r="Y150" s="11" t="n"/>
+      <c r="Z150" s="11" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="11" t="n"/>
@@ -5305,6 +5476,7 @@
       <c r="W151" s="11" t="n"/>
       <c r="X151" s="11" t="n"/>
       <c r="Y151" s="11" t="n"/>
+      <c r="Z151" s="11" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="11" t="n"/>
@@ -5332,6 +5504,7 @@
       <c r="W152" s="11" t="n"/>
       <c r="X152" s="11" t="n"/>
       <c r="Y152" s="11" t="n"/>
+      <c r="Z152" s="11" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="11" t="n"/>
@@ -5359,6 +5532,7 @@
       <c r="W153" s="11" t="n"/>
       <c r="X153" s="11" t="n"/>
       <c r="Y153" s="11" t="n"/>
+      <c r="Z153" s="11" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="11" t="n"/>
@@ -5386,6 +5560,7 @@
       <c r="W154" s="11" t="n"/>
       <c r="X154" s="11" t="n"/>
       <c r="Y154" s="11" t="n"/>
+      <c r="Z154" s="11" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="11" t="n"/>
@@ -5413,6 +5588,7 @@
       <c r="W155" s="11" t="n"/>
       <c r="X155" s="11" t="n"/>
       <c r="Y155" s="11" t="n"/>
+      <c r="Z155" s="11" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="11" t="n"/>
@@ -5440,6 +5616,7 @@
       <c r="W156" s="11" t="n"/>
       <c r="X156" s="11" t="n"/>
       <c r="Y156" s="11" t="n"/>
+      <c r="Z156" s="11" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="11" t="n"/>
@@ -5467,6 +5644,7 @@
       <c r="W157" s="11" t="n"/>
       <c r="X157" s="11" t="n"/>
       <c r="Y157" s="11" t="n"/>
+      <c r="Z157" s="11" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="11" t="n"/>
@@ -5494,6 +5672,7 @@
       <c r="W158" s="11" t="n"/>
       <c r="X158" s="11" t="n"/>
       <c r="Y158" s="11" t="n"/>
+      <c r="Z158" s="11" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="11" t="n"/>
@@ -5521,6 +5700,7 @@
       <c r="W159" s="11" t="n"/>
       <c r="X159" s="11" t="n"/>
       <c r="Y159" s="11" t="n"/>
+      <c r="Z159" s="11" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="11" t="n"/>
@@ -5548,6 +5728,7 @@
       <c r="W160" s="11" t="n"/>
       <c r="X160" s="11" t="n"/>
       <c r="Y160" s="11" t="n"/>
+      <c r="Z160" s="11" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="11" t="n"/>
@@ -5575,6 +5756,7 @@
       <c r="W161" s="11" t="n"/>
       <c r="X161" s="11" t="n"/>
       <c r="Y161" s="11" t="n"/>
+      <c r="Z161" s="11" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="11" t="n"/>
@@ -5602,6 +5784,7 @@
       <c r="W162" s="11" t="n"/>
       <c r="X162" s="11" t="n"/>
       <c r="Y162" s="11" t="n"/>
+      <c r="Z162" s="11" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="11" t="n"/>
@@ -5629,6 +5812,7 @@
       <c r="W163" s="11" t="n"/>
       <c r="X163" s="11" t="n"/>
       <c r="Y163" s="11" t="n"/>
+      <c r="Z163" s="11" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="11" t="n"/>
@@ -5656,6 +5840,7 @@
       <c r="W164" s="11" t="n"/>
       <c r="X164" s="11" t="n"/>
       <c r="Y164" s="11" t="n"/>
+      <c r="Z164" s="11" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="11" t="n"/>
@@ -5683,6 +5868,7 @@
       <c r="W165" s="11" t="n"/>
       <c r="X165" s="11" t="n"/>
       <c r="Y165" s="11" t="n"/>
+      <c r="Z165" s="11" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="11" t="n"/>
@@ -5710,6 +5896,7 @@
       <c r="W166" s="11" t="n"/>
       <c r="X166" s="11" t="n"/>
       <c r="Y166" s="11" t="n"/>
+      <c r="Z166" s="11" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="11" t="n"/>
@@ -5737,6 +5924,7 @@
       <c r="W167" s="11" t="n"/>
       <c r="X167" s="11" t="n"/>
       <c r="Y167" s="11" t="n"/>
+      <c r="Z167" s="11" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="11" t="n"/>
@@ -5764,6 +5952,7 @@
       <c r="W168" s="11" t="n"/>
       <c r="X168" s="11" t="n"/>
       <c r="Y168" s="11" t="n"/>
+      <c r="Z168" s="11" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="11" t="n"/>
@@ -5791,6 +5980,7 @@
       <c r="W169" s="11" t="n"/>
       <c r="X169" s="11" t="n"/>
       <c r="Y169" s="11" t="n"/>
+      <c r="Z169" s="11" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="11" t="n"/>
@@ -5818,6 +6008,7 @@
       <c r="W170" s="11" t="n"/>
       <c r="X170" s="11" t="n"/>
       <c r="Y170" s="11" t="n"/>
+      <c r="Z170" s="11" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="11" t="n"/>
@@ -5845,6 +6036,7 @@
       <c r="W171" s="11" t="n"/>
       <c r="X171" s="11" t="n"/>
       <c r="Y171" s="11" t="n"/>
+      <c r="Z171" s="11" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="11" t="n"/>
@@ -5872,6 +6064,7 @@
       <c r="W172" s="11" t="n"/>
       <c r="X172" s="11" t="n"/>
       <c r="Y172" s="11" t="n"/>
+      <c r="Z172" s="11" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="11" t="n"/>
@@ -5899,6 +6092,7 @@
       <c r="W173" s="11" t="n"/>
       <c r="X173" s="11" t="n"/>
       <c r="Y173" s="11" t="n"/>
+      <c r="Z173" s="11" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="11" t="n"/>
@@ -5926,6 +6120,7 @@
       <c r="W174" s="11" t="n"/>
       <c r="X174" s="11" t="n"/>
       <c r="Y174" s="11" t="n"/>
+      <c r="Z174" s="11" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="11" t="n"/>
@@ -5953,6 +6148,7 @@
       <c r="W175" s="11" t="n"/>
       <c r="X175" s="11" t="n"/>
       <c r="Y175" s="11" t="n"/>
+      <c r="Z175" s="11" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="11" t="n"/>
@@ -5980,6 +6176,7 @@
       <c r="W176" s="11" t="n"/>
       <c r="X176" s="11" t="n"/>
       <c r="Y176" s="11" t="n"/>
+      <c r="Z176" s="11" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="11" t="n"/>
@@ -6007,6 +6204,7 @@
       <c r="W177" s="11" t="n"/>
       <c r="X177" s="11" t="n"/>
       <c r="Y177" s="11" t="n"/>
+      <c r="Z177" s="11" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="11" t="n"/>
@@ -6034,6 +6232,7 @@
       <c r="W178" s="11" t="n"/>
       <c r="X178" s="11" t="n"/>
       <c r="Y178" s="11" t="n"/>
+      <c r="Z178" s="11" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="11" t="n"/>
@@ -6061,6 +6260,7 @@
       <c r="W179" s="11" t="n"/>
       <c r="X179" s="11" t="n"/>
       <c r="Y179" s="11" t="n"/>
+      <c r="Z179" s="11" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="11" t="n"/>
@@ -6088,6 +6288,7 @@
       <c r="W180" s="11" t="n"/>
       <c r="X180" s="11" t="n"/>
       <c r="Y180" s="11" t="n"/>
+      <c r="Z180" s="11" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="11" t="n"/>
@@ -6115,6 +6316,7 @@
       <c r="W181" s="11" t="n"/>
       <c r="X181" s="11" t="n"/>
       <c r="Y181" s="11" t="n"/>
+      <c r="Z181" s="11" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="11" t="n"/>
@@ -6142,6 +6344,7 @@
       <c r="W182" s="11" t="n"/>
       <c r="X182" s="11" t="n"/>
       <c r="Y182" s="11" t="n"/>
+      <c r="Z182" s="11" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="11" t="n"/>
@@ -6169,6 +6372,7 @@
       <c r="W183" s="11" t="n"/>
       <c r="X183" s="11" t="n"/>
       <c r="Y183" s="11" t="n"/>
+      <c r="Z183" s="11" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="11" t="n"/>
@@ -6196,6 +6400,7 @@
       <c r="W184" s="11" t="n"/>
       <c r="X184" s="11" t="n"/>
       <c r="Y184" s="11" t="n"/>
+      <c r="Z184" s="11" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="11" t="n"/>
@@ -6223,6 +6428,7 @@
       <c r="W185" s="11" t="n"/>
       <c r="X185" s="11" t="n"/>
       <c r="Y185" s="11" t="n"/>
+      <c r="Z185" s="11" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="11" t="n"/>
@@ -6250,6 +6456,7 @@
       <c r="W186" s="11" t="n"/>
       <c r="X186" s="11" t="n"/>
       <c r="Y186" s="11" t="n"/>
+      <c r="Z186" s="11" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="11" t="n"/>
@@ -6277,6 +6484,7 @@
       <c r="W187" s="11" t="n"/>
       <c r="X187" s="11" t="n"/>
       <c r="Y187" s="11" t="n"/>
+      <c r="Z187" s="11" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="11" t="n"/>
@@ -6304,6 +6512,7 @@
       <c r="W188" s="11" t="n"/>
       <c r="X188" s="11" t="n"/>
       <c r="Y188" s="11" t="n"/>
+      <c r="Z188" s="11" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="11" t="n"/>
@@ -6331,6 +6540,7 @@
       <c r="W189" s="11" t="n"/>
       <c r="X189" s="11" t="n"/>
       <c r="Y189" s="11" t="n"/>
+      <c r="Z189" s="11" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="11" t="n"/>
@@ -6358,6 +6568,7 @@
       <c r="W190" s="11" t="n"/>
       <c r="X190" s="11" t="n"/>
       <c r="Y190" s="11" t="n"/>
+      <c r="Z190" s="11" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="11" t="n"/>
@@ -6385,6 +6596,7 @@
       <c r="W191" s="11" t="n"/>
       <c r="X191" s="11" t="n"/>
       <c r="Y191" s="11" t="n"/>
+      <c r="Z191" s="11" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="11" t="n"/>
@@ -6412,6 +6624,7 @@
       <c r="W192" s="11" t="n"/>
       <c r="X192" s="11" t="n"/>
       <c r="Y192" s="11" t="n"/>
+      <c r="Z192" s="11" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="11" t="n"/>
@@ -6439,6 +6652,7 @@
       <c r="W193" s="11" t="n"/>
       <c r="X193" s="11" t="n"/>
       <c r="Y193" s="11" t="n"/>
+      <c r="Z193" s="11" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="11" t="n"/>
@@ -6466,6 +6680,7 @@
       <c r="W194" s="11" t="n"/>
       <c r="X194" s="11" t="n"/>
       <c r="Y194" s="11" t="n"/>
+      <c r="Z194" s="11" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="11" t="n"/>
@@ -6493,6 +6708,7 @@
       <c r="W195" s="11" t="n"/>
       <c r="X195" s="11" t="n"/>
       <c r="Y195" s="11" t="n"/>
+      <c r="Z195" s="11" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="11" t="n"/>
@@ -6520,6 +6736,7 @@
       <c r="W196" s="11" t="n"/>
       <c r="X196" s="11" t="n"/>
       <c r="Y196" s="11" t="n"/>
+      <c r="Z196" s="11" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="11" t="n"/>
@@ -6547,6 +6764,7 @@
       <c r="W197" s="11" t="n"/>
       <c r="X197" s="11" t="n"/>
       <c r="Y197" s="11" t="n"/>
+      <c r="Z197" s="11" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="11" t="n"/>
@@ -6574,6 +6792,7 @@
       <c r="W198" s="11" t="n"/>
       <c r="X198" s="11" t="n"/>
       <c r="Y198" s="11" t="n"/>
+      <c r="Z198" s="11" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="11" t="n"/>
@@ -6601,6 +6820,7 @@
       <c r="W199" s="11" t="n"/>
       <c r="X199" s="11" t="n"/>
       <c r="Y199" s="11" t="n"/>
+      <c r="Z199" s="11" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="11" t="n"/>
@@ -6628,6 +6848,7 @@
       <c r="W200" s="11" t="n"/>
       <c r="X200" s="11" t="n"/>
       <c r="Y200" s="11" t="n"/>
+      <c r="Z200" s="11" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="11" t="n"/>
@@ -6655,6 +6876,7 @@
       <c r="W201" s="11" t="n"/>
       <c r="X201" s="11" t="n"/>
       <c r="Y201" s="11" t="n"/>
+      <c r="Z201" s="11" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="11" t="n"/>
@@ -6682,6 +6904,7 @@
       <c r="W202" s="11" t="n"/>
       <c r="X202" s="11" t="n"/>
       <c r="Y202" s="11" t="n"/>
+      <c r="Z202" s="11" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -6691,7 +6914,7 @@
     <dataValidation sqref="E2:E203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid construction status" error="Choose one of: under_construction, ready_to_move" type="list">
       <formula1>"under_construction,ready_to_move"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Z2:Z203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>